<commit_message>
DESKTOP Phase 1: web target boots — RNW installed, web platform config, metro web alias (RNW + Alert shim), browser auth persistence, guarded notifications, system-ui font fallback; expo export --platform web succeeds; phone suite untouched
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-desktop/MK-desktop-audit-v1-2026-08-03.xlsx
+++ b/docs/FCC-desktop/MK-desktop-audit-v1-2026-08-03.xlsx
@@ -544,7 +544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -620,6 +620,40 @@
         </is>
       </c>
     </row>
+    <row r="5" ht="56" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>PHASE 1 STARTED on founder's word ("start building desktop application"). Scaffolding only — no user-facing design before the mock gates.</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="56" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1 milestone: the web build EXPORTS — react-native-web installed; web platform on (metro, single-page); browser dialogs stand in for phone alerts via a web-only module shim (styled sheets come with the design phase); sign-in persistence uses the browser's own storage on web; the notifications side effect is guarded; fonts fall back to the system face. Phone side verified untouched: full suite green.</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Build log</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Desktop audit log: mock v1 delivered, awaiting verdict
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-desktop/MK-desktop-audit-v1-2026-08-03.xlsx
+++ b/docs/FCC-desktop/MK-desktop-audit-v1-2026-08-03.xlsx
@@ -544,7 +544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -654,6 +654,23 @@
         </is>
       </c>
     </row>
+    <row r="7" ht="46" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Desktop mock v1 DELIVERED (mockups/desktop/shell-home-plan-desktop-v1): the sidebar shell + Home + Plan at full width — AWAITING founder verdict. Phase 2 builds nothing until it.</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Awaiting founder</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>